<commit_message>
Version 0.0.2: - improved input/output data format and variable naming; - added dependencies for pyproject.toml; - parameter vector p in the function fitting.bsbcf(), same as in all other routines in the module fitting
</commit_message>
<xml_diff>
--- a/data/dummy_data.xlsx
+++ b/data/dummy_data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\melafit\data\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kolod\projects\melafit\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20787AC2-F947-4730-91FB-C66BB64121A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E5CC90-A765-4B97-AF4A-B49CDDCF2518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{D506D6B8-6E87-4DC8-8544-6572E57FCAF6}"/>
   </bookViews>
@@ -47,10 +47,10 @@
     <t>Mel</t>
   </si>
   <si>
-    <t>Patient</t>
+    <t>Date</t>
   </si>
   <si>
-    <t>Date</t>
+    <t>Participant</t>
   </si>
 </sst>
 </file>
@@ -429,769 +429,769 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
-      </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="1">
-        <v>0.5</v>
+      <c r="A2">
+        <v>1</v>
       </c>
       <c r="B2" s="2">
         <v>46100</v>
       </c>
-      <c r="C2">
-        <v>1</v>
+      <c r="C2" s="1">
+        <v>0.5</v>
       </c>
       <c r="D2">
         <v>1.2</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1">
-        <v>0.625</v>
+      <c r="A3">
+        <v>1</v>
       </c>
       <c r="B3" s="2">
         <v>46100</v>
       </c>
-      <c r="C3">
-        <v>1</v>
+      <c r="C3" s="1">
+        <v>0.625</v>
       </c>
       <c r="D3">
         <v>1.5</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1">
-        <v>0.75</v>
+      <c r="A4">
+        <v>1</v>
       </c>
       <c r="B4" s="2">
         <v>46100</v>
       </c>
-      <c r="C4">
-        <v>1</v>
+      <c r="C4" s="1">
+        <v>0.75</v>
       </c>
       <c r="D4">
         <v>1.8</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="1">
-        <v>0.83333333333333337</v>
+      <c r="A5">
+        <v>1</v>
       </c>
       <c r="B5" s="2">
         <v>46100</v>
       </c>
-      <c r="C5">
-        <v>1</v>
+      <c r="C5" s="1">
+        <v>0.83333333333333337</v>
       </c>
       <c r="D5">
         <v>2.1</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1">
-        <v>0.875</v>
+      <c r="A6">
+        <v>1</v>
       </c>
       <c r="B6" s="2">
         <v>46100</v>
       </c>
-      <c r="C6">
-        <v>1</v>
+      <c r="C6" s="1">
+        <v>0.875</v>
       </c>
       <c r="D6">
         <v>9.4</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="1">
-        <v>0.91666666666666663</v>
+      <c r="A7">
+        <v>1</v>
       </c>
       <c r="B7" s="2">
         <v>46100</v>
       </c>
-      <c r="C7">
-        <v>1</v>
+      <c r="C7" s="1">
+        <v>0.91666666666666663</v>
       </c>
       <c r="D7">
         <v>28.5</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1">
-        <v>0.95833333333333337</v>
+      <c r="A8">
+        <v>1</v>
       </c>
       <c r="B8" s="2">
         <v>46100</v>
       </c>
-      <c r="C8">
-        <v>1</v>
+      <c r="C8" s="1">
+        <v>0.95833333333333337</v>
       </c>
       <c r="D8">
         <v>46.2</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>0</v>
+      <c r="A9">
+        <v>1</v>
       </c>
       <c r="B9" s="2">
         <v>46101</v>
       </c>
-      <c r="C9">
-        <v>1</v>
+      <c r="C9" s="1">
+        <v>0</v>
       </c>
       <c r="D9">
         <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1">
-        <v>4.1666666666666664E-2</v>
+      <c r="A10">
+        <v>1</v>
       </c>
       <c r="B10" s="2">
         <v>46101</v>
       </c>
-      <c r="C10">
-        <v>1</v>
+      <c r="C10" s="1">
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D10">
         <v>51.5</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1">
-        <v>8.3333333333333329E-2</v>
+      <c r="A11">
+        <v>1</v>
       </c>
       <c r="B11" s="2">
         <v>46101</v>
       </c>
-      <c r="C11">
-        <v>1</v>
+      <c r="C11" s="1">
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="D11">
         <v>50.2</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1">
-        <v>0.125</v>
+      <c r="A12">
+        <v>1</v>
       </c>
       <c r="B12" s="2">
         <v>46101</v>
       </c>
-      <c r="C12">
-        <v>1</v>
+      <c r="C12" s="1">
+        <v>0.125</v>
       </c>
       <c r="D12">
         <v>47.5</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1">
-        <v>0.16666666666666666</v>
+      <c r="A13">
+        <v>1</v>
       </c>
       <c r="B13" s="2">
         <v>46101</v>
       </c>
-      <c r="C13">
-        <v>1</v>
+      <c r="C13" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="D13">
         <v>43.8</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1">
-        <v>0.20833333333333334</v>
+      <c r="A14">
+        <v>1</v>
       </c>
       <c r="B14" s="2">
         <v>46101</v>
       </c>
-      <c r="C14">
-        <v>1</v>
+      <c r="C14" s="1">
+        <v>0.20833333333333334</v>
       </c>
       <c r="D14">
         <v>37.5</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1">
-        <v>0.25</v>
+      <c r="A15">
+        <v>1</v>
       </c>
       <c r="B15" s="2">
         <v>46101</v>
       </c>
-      <c r="C15">
-        <v>1</v>
+      <c r="C15" s="1">
+        <v>0.25</v>
       </c>
       <c r="D15">
         <v>29.8</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1">
-        <v>0.29166666666666669</v>
+      <c r="A16">
+        <v>1</v>
       </c>
       <c r="B16" s="2">
         <v>46101</v>
       </c>
-      <c r="C16">
-        <v>1</v>
+      <c r="C16" s="1">
+        <v>0.29166666666666669</v>
       </c>
       <c r="D16">
         <v>21.8</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="1">
-        <v>0.33333333333333331</v>
+      <c r="A17">
+        <v>1</v>
       </c>
       <c r="B17" s="2">
         <v>46101</v>
       </c>
-      <c r="C17">
-        <v>1</v>
+      <c r="C17" s="1">
+        <v>0.33333333333333331</v>
       </c>
       <c r="D17">
         <v>8.8000000000000007</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="1">
-        <v>0.375</v>
+      <c r="A18">
+        <v>1</v>
       </c>
       <c r="B18" s="2">
         <v>46101</v>
       </c>
-      <c r="C18">
-        <v>1</v>
+      <c r="C18" s="1">
+        <v>0.375</v>
       </c>
       <c r="D18">
         <v>2.4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="1">
-        <v>0.5</v>
+      <c r="A19">
+        <v>1</v>
       </c>
       <c r="B19" s="2">
         <v>46101</v>
       </c>
-      <c r="C19">
-        <v>1</v>
+      <c r="C19" s="1">
+        <v>0.5</v>
       </c>
       <c r="D19">
         <v>1.2</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1">
-        <v>0.5</v>
+      <c r="A20">
+        <v>2</v>
       </c>
       <c r="B20" s="2">
         <v>46102</v>
       </c>
-      <c r="C20">
-        <v>2</v>
+      <c r="C20" s="1">
+        <v>0.5</v>
       </c>
       <c r="D20">
         <v>1.8</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1">
-        <v>0.625</v>
+      <c r="A21">
+        <v>2</v>
       </c>
       <c r="B21" s="2">
         <v>46102</v>
       </c>
-      <c r="C21">
-        <v>2</v>
+      <c r="C21" s="1">
+        <v>0.625</v>
       </c>
       <c r="D21">
         <v>2.1</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
-        <v>0.75</v>
+      <c r="A22">
+        <v>2</v>
       </c>
       <c r="B22" s="2">
         <v>46102</v>
       </c>
-      <c r="C22">
-        <v>2</v>
+      <c r="C22" s="1">
+        <v>0.75</v>
       </c>
       <c r="D22">
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
-        <v>0.83333333333333337</v>
+      <c r="A23">
+        <v>2</v>
       </c>
       <c r="B23" s="2">
         <v>46102</v>
       </c>
-      <c r="C23">
-        <v>2</v>
+      <c r="C23" s="1">
+        <v>0.83333333333333337</v>
       </c>
       <c r="D23">
         <v>4.8</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>0.875</v>
+      <c r="A24">
+        <v>2</v>
       </c>
       <c r="B24" s="2">
         <v>46102</v>
       </c>
-      <c r="C24">
-        <v>2</v>
+      <c r="C24" s="1">
+        <v>0.875</v>
       </c>
       <c r="D24">
         <v>14.5</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>0.91666666666666663</v>
+      <c r="A25">
+        <v>2</v>
       </c>
       <c r="B25" s="2">
         <v>46102</v>
       </c>
-      <c r="C25">
-        <v>2</v>
+      <c r="C25" s="1">
+        <v>0.91666666666666663</v>
       </c>
       <c r="D25">
         <v>44</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>0.95833333333333337</v>
+      <c r="A26">
+        <v>2</v>
       </c>
       <c r="B26" s="2">
         <v>46102</v>
       </c>
-      <c r="C26">
-        <v>2</v>
+      <c r="C26" s="1">
+        <v>0.95833333333333337</v>
       </c>
       <c r="D26">
         <v>64.2</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
-        <v>0</v>
+      <c r="A27">
+        <v>2</v>
       </c>
       <c r="B27" s="2">
         <v>46103</v>
       </c>
-      <c r="C27">
-        <v>2</v>
+      <c r="C27" s="1">
+        <v>0</v>
       </c>
       <c r="D27">
         <v>79.5</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
-        <v>4.1666666666666664E-2</v>
+      <c r="A28">
+        <v>2</v>
       </c>
       <c r="B28" s="2">
         <v>46103</v>
       </c>
-      <c r="C28">
-        <v>2</v>
+      <c r="C28" s="1">
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D28">
         <v>83.2</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>8.3333333333333329E-2</v>
+      <c r="A29">
+        <v>2</v>
       </c>
       <c r="B29" s="2">
         <v>46103</v>
       </c>
-      <c r="C29">
-        <v>2</v>
+      <c r="C29" s="1">
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="D29">
         <v>81.5</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>0.125</v>
+      <c r="A30">
+        <v>2</v>
       </c>
       <c r="B30" s="2">
         <v>46103</v>
       </c>
-      <c r="C30">
-        <v>2</v>
+      <c r="C30" s="1">
+        <v>0.125</v>
       </c>
       <c r="D30">
         <v>77.2</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>0.16666666666666666</v>
+      <c r="A31">
+        <v>2</v>
       </c>
       <c r="B31" s="2">
         <v>46103</v>
       </c>
-      <c r="C31">
-        <v>2</v>
+      <c r="C31" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="D31">
         <v>76.5</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
-        <v>0.20833333333333334</v>
+      <c r="A32">
+        <v>2</v>
       </c>
       <c r="B32" s="2">
         <v>46103</v>
       </c>
-      <c r="C32">
-        <v>2</v>
+      <c r="C32" s="1">
+        <v>0.20833333333333334</v>
       </c>
       <c r="D32">
         <v>79.2</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
-        <v>0.25</v>
+      <c r="A33">
+        <v>2</v>
       </c>
       <c r="B33" s="2">
         <v>46103</v>
       </c>
-      <c r="C33">
-        <v>2</v>
+      <c r="C33" s="1">
+        <v>0.25</v>
       </c>
       <c r="D33">
         <v>65.5</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>0.29166666666666669</v>
+      <c r="A34">
+        <v>2</v>
       </c>
       <c r="B34" s="2">
         <v>46103</v>
       </c>
-      <c r="C34">
-        <v>2</v>
+      <c r="C34" s="1">
+        <v>0.29166666666666669</v>
       </c>
       <c r="D34">
         <v>44.5</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>0.33333333333333331</v>
+      <c r="A35">
+        <v>2</v>
       </c>
       <c r="B35" s="2">
         <v>46103</v>
       </c>
-      <c r="C35">
-        <v>2</v>
+      <c r="C35" s="1">
+        <v>0.33333333333333331</v>
       </c>
       <c r="D35">
         <v>15.5</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>0.375</v>
+      <c r="A36">
+        <v>2</v>
       </c>
       <c r="B36" s="2">
         <v>46103</v>
       </c>
-      <c r="C36">
-        <v>2</v>
+      <c r="C36" s="1">
+        <v>0.375</v>
       </c>
       <c r="D36">
         <v>5.2</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
-        <v>0.5</v>
+      <c r="A37">
+        <v>2</v>
       </c>
       <c r="B37" s="2">
         <v>46103</v>
       </c>
-      <c r="C37">
-        <v>2</v>
+      <c r="C37" s="1">
+        <v>0.5</v>
       </c>
       <c r="D37">
         <v>1.9</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
-        <v>0.5</v>
+      <c r="A38">
+        <v>3</v>
       </c>
       <c r="B38" s="2">
         <v>46104</v>
       </c>
-      <c r="C38">
-        <v>3</v>
+      <c r="C38" s="1">
+        <v>0.5</v>
       </c>
       <c r="D38">
         <v>2.1</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>0.625</v>
+      <c r="A39">
+        <v>3</v>
       </c>
       <c r="B39" s="2">
         <v>46104</v>
       </c>
-      <c r="C39">
-        <v>3</v>
+      <c r="C39" s="1">
+        <v>0.625</v>
       </c>
       <c r="D39">
         <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <v>0.75</v>
+      <c r="A40">
+        <v>3</v>
       </c>
       <c r="B40" s="2">
         <v>46104</v>
       </c>
-      <c r="C40">
-        <v>3</v>
+      <c r="C40" s="1">
+        <v>0.75</v>
       </c>
       <c r="D40">
         <v>2.5</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>0.83333333333333337</v>
+      <c r="A41">
+        <v>3</v>
       </c>
       <c r="B41" s="2">
         <v>46104</v>
       </c>
-      <c r="C41">
-        <v>3</v>
+      <c r="C41" s="1">
+        <v>0.83333333333333337</v>
       </c>
       <c r="D41">
         <v>5.2</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="1">
-        <v>0.875</v>
+      <c r="A42">
+        <v>3</v>
       </c>
       <c r="B42" s="2">
         <v>46104</v>
       </c>
-      <c r="C42">
-        <v>3</v>
+      <c r="C42" s="1">
+        <v>0.875</v>
       </c>
       <c r="D42">
         <v>11</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="1">
-        <v>0.91666666666666663</v>
+      <c r="A43">
+        <v>3</v>
       </c>
       <c r="B43" s="2">
         <v>46104</v>
       </c>
-      <c r="C43">
-        <v>3</v>
+      <c r="C43" s="1">
+        <v>0.91666666666666663</v>
       </c>
       <c r="D43">
         <v>20.2</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="1">
-        <v>0.95833333333333337</v>
+      <c r="A44">
+        <v>3</v>
       </c>
       <c r="B44" s="2">
         <v>46104</v>
       </c>
-      <c r="C44">
-        <v>3</v>
+      <c r="C44" s="1">
+        <v>0.95833333333333337</v>
       </c>
       <c r="D44">
         <v>34.799999999999997</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="1">
-        <v>0</v>
+      <c r="A45">
+        <v>3</v>
       </c>
       <c r="B45" s="2">
         <v>46105</v>
       </c>
-      <c r="C45">
-        <v>3</v>
+      <c r="C45" s="1">
+        <v>0</v>
       </c>
       <c r="D45">
         <v>45.5</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="1">
-        <v>4.1666666666666664E-2</v>
+      <c r="A46">
+        <v>3</v>
       </c>
       <c r="B46" s="2">
         <v>46105</v>
       </c>
-      <c r="C46">
-        <v>3</v>
+      <c r="C46" s="1">
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D46">
         <v>58.2</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="1">
-        <v>8.3333333333333329E-2</v>
+      <c r="A47">
+        <v>3</v>
       </c>
       <c r="B47" s="2">
         <v>46105</v>
       </c>
-      <c r="C47">
-        <v>3</v>
+      <c r="C47" s="1">
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="D47">
         <v>52.8</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="1">
-        <v>0.125</v>
+      <c r="A48">
+        <v>3</v>
       </c>
       <c r="B48" s="2">
         <v>46105</v>
       </c>
-      <c r="C48">
-        <v>3</v>
+      <c r="C48" s="1">
+        <v>0.125</v>
       </c>
       <c r="D48">
         <v>57.5</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="1">
-        <v>0.16666666666666666</v>
+      <c r="A49">
+        <v>3</v>
       </c>
       <c r="B49" s="2">
         <v>46105</v>
       </c>
-      <c r="C49">
-        <v>3</v>
+      <c r="C49" s="1">
+        <v>0.16666666666666666</v>
       </c>
       <c r="D49">
         <v>61.8</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A50" s="1">
-        <v>0.20833333333333334</v>
+      <c r="A50">
+        <v>3</v>
       </c>
       <c r="B50" s="2">
         <v>46105</v>
       </c>
-      <c r="C50">
-        <v>3</v>
+      <c r="C50" s="1">
+        <v>0.20833333333333334</v>
       </c>
       <c r="D50">
         <v>54.2</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A51" s="1">
-        <v>0.25</v>
+      <c r="A51">
+        <v>3</v>
       </c>
       <c r="B51" s="2">
         <v>46105</v>
       </c>
-      <c r="C51">
-        <v>3</v>
+      <c r="C51" s="1">
+        <v>0.25</v>
       </c>
       <c r="D51">
         <v>42.5</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A52" s="1">
-        <v>0.29166666666666669</v>
+      <c r="A52">
+        <v>3</v>
       </c>
       <c r="B52" s="2">
         <v>46105</v>
       </c>
-      <c r="C52">
-        <v>3</v>
+      <c r="C52" s="1">
+        <v>0.29166666666666669</v>
       </c>
       <c r="D52">
         <v>31.2</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A53" s="1">
-        <v>0.33333333333333331</v>
+      <c r="A53">
+        <v>3</v>
       </c>
       <c r="B53" s="2">
         <v>46105</v>
       </c>
-      <c r="C53">
-        <v>3</v>
+      <c r="C53" s="1">
+        <v>0.33333333333333331</v>
       </c>
       <c r="D53">
         <v>10.5</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A54" s="1">
-        <v>0.375</v>
+      <c r="A54">
+        <v>3</v>
       </c>
       <c r="B54" s="2">
         <v>46105</v>
       </c>
-      <c r="C54">
-        <v>3</v>
+      <c r="C54" s="1">
+        <v>0.375</v>
       </c>
       <c r="D54">
         <v>3.2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A55" s="1">
-        <v>0.5</v>
+      <c r="A55">
+        <v>3</v>
       </c>
       <c r="B55" s="2">
         <v>46105</v>
       </c>
-      <c r="C55">
-        <v>3</v>
+      <c r="C55" s="1">
+        <v>0.5</v>
       </c>
       <c r="D55">
         <v>2.2000000000000002</v>

</xml_diff>